<commit_message>
Excel3 FK 예제 샘플 추가 (School/Teacher/Student)
</commit_message>
<xml_diff>
--- a/Docs/SampleExcels/Excel3.xlsx
+++ b/Docs/SampleExcels/Excel3.xlsx
@@ -5,10 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="School" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Teacher" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Student" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
   <si>
     <t xml:space="preserve">C7</t>
   </si>
@@ -170,6 +172,42 @@
   </si>
   <si>
     <t xml:space="preserve">Естественные</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SchoolName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김민준</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이서연</t>
+  </si>
+  <si>
+    <t xml:space="preserve">박지호</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SchoolId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TeacherId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">최아름</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정우진</t>
+  </si>
+  <si>
+    <t xml:space="preserve">한소희</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오민재</t>
+  </si>
+  <si>
+    <t xml:space="preserve">윤채원</t>
   </si>
 </sst>
 </file>
@@ -760,4 +798,190 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff페이지 &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff페이지 &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>